<commit_message>
[IMP] python task-1 file.
</commit_message>
<xml_diff>
--- a/python_test/sale_data.xlsx
+++ b/python_test/sale_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,11 @@
           <t>quantity</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SubTotal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -467,6 +472,9 @@
       <c r="D2" t="n">
         <v>8</v>
       </c>
+      <c r="E2" t="n">
+        <v>1480</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -485,6 +493,9 @@
       <c r="D3" t="n">
         <v>10</v>
       </c>
+      <c r="E3" t="n">
+        <v>3860</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +514,9 @@
       <c r="D4" t="n">
         <v>4</v>
       </c>
+      <c r="E4" t="n">
+        <v>848</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -521,6 +535,9 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
+      <c r="E5" t="n">
+        <v>951</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -539,6 +556,9 @@
       <c r="D6" t="n">
         <v>9</v>
       </c>
+      <c r="E6" t="n">
+        <v>3573</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -557,6 +577,9 @@
       <c r="D7" t="n">
         <v>9</v>
       </c>
+      <c r="E7" t="n">
+        <v>5409</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -575,6 +598,9 @@
       <c r="D8" t="n">
         <v>5</v>
       </c>
+      <c r="E8" t="n">
+        <v>3765</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -593,6 +619,9 @@
       <c r="D9" t="n">
         <v>9</v>
       </c>
+      <c r="E9" t="n">
+        <v>2808</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -611,6 +640,9 @@
       <c r="D10" t="n">
         <v>8</v>
       </c>
+      <c r="E10" t="n">
+        <v>3056</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -629,6 +661,9 @@
       <c r="D11" t="n">
         <v>1</v>
       </c>
+      <c r="E11" t="n">
+        <v>512</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -647,6 +682,9 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
+      <c r="E12" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -665,6 +703,9 @@
       <c r="D13" t="n">
         <v>4</v>
       </c>
+      <c r="E13" t="n">
+        <v>3636</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -683,6 +724,9 @@
       <c r="D14" t="n">
         <v>10</v>
       </c>
+      <c r="E14" t="n">
+        <v>5770</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -701,6 +745,9 @@
       <c r="D15" t="n">
         <v>6</v>
       </c>
+      <c r="E15" t="n">
+        <v>1254</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -719,6 +766,9 @@
       <c r="D16" t="n">
         <v>10</v>
       </c>
+      <c r="E16" t="n">
+        <v>8120</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -737,6 +787,9 @@
       <c r="D17" t="n">
         <v>5</v>
       </c>
+      <c r="E17" t="n">
+        <v>805</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -755,6 +808,9 @@
       <c r="D18" t="n">
         <v>2</v>
       </c>
+      <c r="E18" t="n">
+        <v>1254</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -773,6 +829,9 @@
       <c r="D19" t="n">
         <v>9</v>
       </c>
+      <c r="E19" t="n">
+        <v>8118</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -791,6 +850,9 @@
       <c r="D20" t="n">
         <v>4</v>
       </c>
+      <c r="E20" t="n">
+        <v>3676</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -809,6 +871,9 @@
       <c r="D21" t="n">
         <v>10</v>
       </c>
+      <c r="E21" t="n">
+        <v>4040</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -827,6 +892,9 @@
       <c r="D22" t="n">
         <v>7</v>
       </c>
+      <c r="E22" t="n">
+        <v>1155</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -845,6 +913,9 @@
       <c r="D23" t="n">
         <v>1</v>
       </c>
+      <c r="E23" t="n">
+        <v>782</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -863,6 +934,9 @@
       <c r="D24" t="n">
         <v>4</v>
       </c>
+      <c r="E24" t="n">
+        <v>3592</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -881,6 +955,9 @@
       <c r="D25" t="n">
         <v>8</v>
       </c>
+      <c r="E25" t="n">
+        <v>7456</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -899,6 +976,9 @@
       <c r="D26" t="n">
         <v>6</v>
       </c>
+      <c r="E26" t="n">
+        <v>1278</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -917,6 +997,9 @@
       <c r="D27" t="n">
         <v>2</v>
       </c>
+      <c r="E27" t="n">
+        <v>1736</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -935,6 +1018,9 @@
       <c r="D28" t="n">
         <v>4</v>
       </c>
+      <c r="E28" t="n">
+        <v>1856</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -953,6 +1039,9 @@
       <c r="D29" t="n">
         <v>6</v>
       </c>
+      <c r="E29" t="n">
+        <v>4584</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -971,6 +1060,9 @@
       <c r="D30" t="n">
         <v>9</v>
       </c>
+      <c r="E30" t="n">
+        <v>4779</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -988,6 +1080,9 @@
       </c>
       <c r="D31" t="n">
         <v>5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3050</v>
       </c>
     </row>
   </sheetData>

</xml_diff>